<commit_message>
fix(compliance): complete Section 22.5 relocation response in Anchor questionnaire
</commit_message>
<xml_diff>
--- a/documents/Anchor Submission Package/01 - Anchor Onboarding Questionnaire.xlsx
+++ b/documents/Anchor Submission Package/01 - Anchor Onboarding Questionnaire.xlsx
@@ -516,7 +516,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -743,7 +743,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -3510,7 +3509,7 @@
       </c>
       <c r="C68" s="25" t="inlineStr">
         <is>
-          <t>Yes, provided compliance status remains active and ongoing KYC requirements are fulfilled.</t>
+          <t>Yes, subject to full KYC verification (valid Nigerian residency permit, alien registration, international passport, and proof of address).</t>
         </is>
       </c>
       <c r="D68" s="4" t="n"/>
@@ -3544,7 +3543,11 @@
           <t>Would this customer be allowed to continue using the account if they no longer reside in Nigera ?</t>
         </is>
       </c>
-      <c r="C69" s="84" t="n"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Yes, subject to ongoing compliance requirements. Existing customers who relocate outside Nigeria may continue using eligible services after completing any required KYC refresh, sanctions screening, and regulatory checks. Services restricted by applicable laws, regulatory requirements, or provider availability may be limited or suspended depending on the customer's country of residence.</t>
+        </is>
+      </c>
       <c r="D69" s="4" t="n"/>
       <c r="E69" s="4" t="n"/>
       <c r="F69" s="4" t="n"/>
@@ -4759,7 +4762,7 @@
       <c r="Z102" s="4" t="n"/>
     </row>
     <row r="103" ht="15.75" customHeight="1" s="79">
-      <c r="A103" s="85" t="n"/>
+      <c r="A103" s="84" t="n"/>
       <c r="B103" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve"> -     Customers</t>
@@ -4795,7 +4798,7 @@
       <c r="Z103" s="4" t="n"/>
     </row>
     <row r="104" ht="15.75" customHeight="1" s="79">
-      <c r="A104" s="85" t="n"/>
+      <c r="A104" s="84" t="n"/>
       <c r="B104" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve"> -     Employees</t>
@@ -4831,7 +4834,7 @@
       <c r="Z104" s="4" t="n"/>
     </row>
     <row r="105" ht="15.75" customHeight="1" s="79">
-      <c r="A105" s="86" t="n"/>
+      <c r="A105" s="85" t="n"/>
       <c r="B105" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve"> -     Contractors</t>
@@ -5823,14 +5826,13 @@
       <c r="Z131" s="43" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="11">
     <mergeCell ref="A102:A105"/>
     <mergeCell ref="A89:A101"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A83:A88"/>
     <mergeCell ref="A51:A52"/>
     <mergeCell ref="A55:A56"/>
-    <mergeCell ref="C68:C69"/>
     <mergeCell ref="A36:A44"/>
     <mergeCell ref="A22:A33"/>
     <mergeCell ref="A76:A82"/>

</xml_diff>